<commit_message>
added polygon cutout under RF connector
updated fab files
</commit_message>
<xml_diff>
--- a/GPS-Module-PCB/Fabrication files/Fab File V1/Bill of Materials for GPS-MINI-V1-2025-10-31.xlsx
+++ b/GPS-Module-PCB/Fabrication files/Fab File V1/Bill of Materials for GPS-MINI-V1-2025-10-31.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\QRBOTS\PCB Projects\GPS_Mini_Only\GPS-Module-PCB\Fabrication files\Fab File V1\Fabrication V1\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\QRBOTS\PCB Projects\GPS_Mini_Only\GPS-Module-PCB\Fabrication files\Fab File V1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E4BA222-6706-42BA-8C63-0298A48ED3E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38B6EF59-BD7C-43EC-9EF1-ECC44CD13ECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="110">
   <si>
     <t>Source Data From:</t>
   </si>
@@ -92,9 +92,6 @@
     <t>C6</t>
   </si>
   <si>
-    <t>C9, C10</t>
-  </si>
-  <si>
     <t>D1</t>
   </si>
   <si>
@@ -155,9 +152,6 @@
     <t>U4</t>
   </si>
   <si>
-    <t>U5</t>
-  </si>
-  <si>
     <t>U6</t>
   </si>
   <si>
@@ -185,9 +179,6 @@
     <t>Multilayer Ceramic Capacitor, CC Series, 4.7 - F, - 10%, X5R, 6.3 V, 0603 [1608 Metric]</t>
   </si>
   <si>
-    <t>0402 10000 pF 16 V ±10% Tolerance X7R Multilayer Ceramic Chip Capacitor, Multilayer Ceramic Capacitors MLCC - SMD/SMT 25V 0.01uF X7R 0402 10%</t>
-  </si>
-  <si>
     <t>TVS DIODE 14VWM 40VC 0402</t>
   </si>
   <si>
@@ -248,9 +239,6 @@
     <t>TVS DIODE 5VWM 10VC 10UDFN</t>
   </si>
   <si>
-    <t>series RF Receiver BeiDou, Galileo, GLONASS, GNSS, GPS 1.207GHz, 1.2276GHz, 1.246GHz, 1.561GHz, 1.575GHz, 1.602GHz -167dBm 921.6kbps - 54-LGA (22x17)</t>
-  </si>
-  <si>
     <t>Automotive 3-ch, 1.65-V to 5.5-V buffers with open-drain outputs 8-VSSOP -40 to 125</t>
   </si>
   <si>
@@ -278,9 +266,6 @@
     <t>CC0603KRX5R5BB475</t>
   </si>
   <si>
-    <t>GRM155R71C103KA01D, C0402C103K3REC7411</t>
-  </si>
-  <si>
     <t>PESD0402-140</t>
   </si>
   <si>
@@ -341,9 +326,6 @@
     <t>ESD7104MUTAG</t>
   </si>
   <si>
-    <t>ZED-F9P-04B</t>
-  </si>
-  <si>
     <t>SN74LVC3G07QDCURQ1</t>
   </si>
   <si>
@@ -363,6 +345,24 @@
   </si>
   <si>
     <t>GPS-Module-New.BomDoc</t>
+  </si>
+  <si>
+    <t>C9</t>
+  </si>
+  <si>
+    <t>C10</t>
+  </si>
+  <si>
+    <t>0402 10000 pF 16 V ±10% Tolerance X7R Multilayer Ceramic Chip Capacitor</t>
+  </si>
+  <si>
+    <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 25V 0.01uF X7R 0402 10%</t>
+  </si>
+  <si>
+    <t>GRM155R71C103KA01D</t>
+  </si>
+  <si>
+    <t>C0402C103K3REC7411</t>
   </si>
 </sst>
 </file>
@@ -1264,7 +1264,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J97"/>
+  <dimension ref="A1:J95"/>
   <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.5546875" style="2" customWidth="1"/>
@@ -1299,7 +1299,7 @@
       <c r="D2" s="69"/>
       <c r="E2" s="70"/>
       <c r="F2" s="38" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G2" s="39"/>
       <c r="H2" s="37"/>
@@ -1315,7 +1315,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="40" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="G3" s="41"/>
       <c r="H3" s="33"/>
@@ -1331,7 +1331,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="G4" s="43"/>
       <c r="H4" s="28"/>
@@ -1374,7 +1374,7 @@
         <v>12</v>
       </c>
       <c r="E7" s="26">
-        <v>45958</v>
+        <v>45961</v>
       </c>
       <c r="F7" s="5"/>
       <c r="G7" s="46"/>
@@ -1390,7 +1390,7 @@
         <v>13</v>
       </c>
       <c r="E8" s="27">
-        <v>45958</v>
+        <v>45961</v>
       </c>
       <c r="F8" s="9"/>
       <c r="G8" s="46"/>
@@ -1424,18 +1424,18 @@
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
       <c r="B10" s="52"/>
-      <c r="C10" s="63">
+      <c r="C10" s="57">
         <v>1</v>
       </c>
       <c r="D10" s="58" t="s">
         <v>14</v>
       </c>
       <c r="E10" s="58" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F10" s="25"/>
       <c r="G10" s="58" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="H10" s="35"/>
       <c r="I10"/>
@@ -1443,18 +1443,18 @@
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="10"/>
       <c r="B11" s="52"/>
-      <c r="C11" s="63">
+      <c r="C11" s="57">
         <v>2</v>
       </c>
       <c r="D11" s="58" t="s">
         <v>15</v>
       </c>
       <c r="E11" s="58" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F11" s="25"/>
       <c r="G11" s="58" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="H11" s="35"/>
       <c r="I11"/>
@@ -1464,18 +1464,18 @@
         <v>3</v>
       </c>
       <c r="B12" s="51"/>
-      <c r="C12" s="63">
+      <c r="C12" s="57">
         <v>5</v>
       </c>
       <c r="D12" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E12" s="58" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F12" s="25"/>
       <c r="G12" s="58" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H12" s="35"/>
       <c r="I12"/>
@@ -1485,18 +1485,18 @@
         <v>3</v>
       </c>
       <c r="B13" s="52"/>
-      <c r="C13" s="63">
+      <c r="C13" s="57">
         <v>2</v>
       </c>
       <c r="D13" s="58" t="s">
         <v>17</v>
       </c>
       <c r="E13" s="58" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F13" s="25"/>
       <c r="G13" s="58" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H13" s="35"/>
       <c r="I13"/>
@@ -1506,18 +1506,18 @@
         <v>3</v>
       </c>
       <c r="B14" s="52"/>
-      <c r="C14" s="63">
+      <c r="C14" s="57">
         <v>1</v>
       </c>
       <c r="D14" s="58" t="s">
         <v>18</v>
       </c>
       <c r="E14" s="58" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F14" s="25"/>
       <c r="G14" s="58" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="H14" s="35"/>
       <c r="I14"/>
@@ -1527,18 +1527,18 @@
         <v>3</v>
       </c>
       <c r="B15" s="51"/>
-      <c r="C15" s="63">
-        <v>2</v>
+      <c r="C15" s="57">
+        <v>1</v>
       </c>
       <c r="D15" s="58" t="s">
-        <v>19</v>
+        <v>104</v>
       </c>
       <c r="E15" s="58" t="s">
-        <v>50</v>
+        <v>106</v>
       </c>
       <c r="F15" s="25"/>
       <c r="G15" s="58" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="H15" s="35"/>
       <c r="I15"/>
@@ -1548,18 +1548,18 @@
         <v>3</v>
       </c>
       <c r="B16" s="52"/>
-      <c r="C16" s="63">
+      <c r="C16" s="57">
         <v>1</v>
       </c>
       <c r="D16" s="58" t="s">
-        <v>20</v>
+        <v>105</v>
       </c>
       <c r="E16" s="58" t="s">
-        <v>51</v>
+        <v>107</v>
       </c>
       <c r="F16" s="25"/>
       <c r="G16" s="58" t="s">
-        <v>82</v>
+        <v>109</v>
       </c>
       <c r="H16" s="35"/>
       <c r="I16"/>
@@ -1569,18 +1569,18 @@
         <v>3</v>
       </c>
       <c r="B17" s="51"/>
-      <c r="C17" s="63">
+      <c r="C17" s="57">
         <v>1</v>
       </c>
       <c r="D17" s="58" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E17" s="58" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F17" s="25"/>
       <c r="G17" s="58" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="H17" s="35"/>
       <c r="I17"/>
@@ -1590,18 +1590,18 @@
         <v>3</v>
       </c>
       <c r="B18" s="52"/>
-      <c r="C18" s="63">
+      <c r="C18" s="57">
         <v>1</v>
       </c>
       <c r="D18" s="58" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E18" s="58" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F18" s="25"/>
       <c r="G18" s="58" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="H18" s="35"/>
       <c r="I18"/>
@@ -1610,19 +1610,19 @@
       <c r="A19" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B19" s="52"/>
-      <c r="C19" s="63">
+      <c r="B19" s="51"/>
+      <c r="C19" s="57">
         <v>1</v>
       </c>
       <c r="D19" s="58" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E19" s="58" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F19" s="25"/>
       <c r="G19" s="58" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="H19" s="35"/>
       <c r="I19"/>
@@ -1631,19 +1631,19 @@
       <c r="A20" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B20" s="51"/>
-      <c r="C20" s="63">
+      <c r="B20" s="52"/>
+      <c r="C20" s="57">
         <v>1</v>
       </c>
       <c r="D20" s="58" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E20" s="58" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F20" s="25"/>
       <c r="G20" s="58" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="H20" s="35"/>
       <c r="I20"/>
@@ -1653,18 +1653,18 @@
         <v>3</v>
       </c>
       <c r="B21" s="52"/>
-      <c r="C21" s="63">
+      <c r="C21" s="57">
         <v>1</v>
       </c>
       <c r="D21" s="58" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E21" s="58" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F21" s="25"/>
       <c r="G21" s="58" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="H21" s="35"/>
       <c r="I21"/>
@@ -1673,19 +1673,19 @@
       <c r="A22" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B22" s="52"/>
-      <c r="C22" s="63">
+      <c r="B22" s="51"/>
+      <c r="C22" s="57">
         <v>1</v>
       </c>
       <c r="D22" s="58" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E22" s="58" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F22" s="25"/>
       <c r="G22" s="58" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="H22" s="35"/>
       <c r="I22"/>
@@ -1694,19 +1694,19 @@
       <c r="A23" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B23" s="51"/>
-      <c r="C23" s="63">
+      <c r="B23" s="52"/>
+      <c r="C23" s="57">
         <v>1</v>
       </c>
       <c r="D23" s="58" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E23" s="58" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F23" s="25"/>
       <c r="G23" s="58" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="H23" s="35"/>
       <c r="I23"/>
@@ -1715,19 +1715,19 @@
       <c r="A24" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B24" s="52"/>
-      <c r="C24" s="63">
-        <v>2</v>
+      <c r="B24" s="51"/>
+      <c r="C24" s="57">
+        <v>1</v>
       </c>
       <c r="D24" s="58" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E24" s="58" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F24" s="25"/>
       <c r="G24" s="58" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="H24" s="35"/>
       <c r="I24"/>
@@ -1736,19 +1736,19 @@
       <c r="A25" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B25" s="51"/>
-      <c r="C25" s="63">
+      <c r="B25" s="52"/>
+      <c r="C25" s="57">
         <v>2</v>
       </c>
       <c r="D25" s="58" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E25" s="58" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F25" s="25"/>
       <c r="G25" s="58" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="H25" s="35"/>
       <c r="I25"/>
@@ -1758,18 +1758,18 @@
         <v>3</v>
       </c>
       <c r="B26" s="52"/>
-      <c r="C26" s="63">
-        <v>3</v>
+      <c r="C26" s="57">
+        <v>2</v>
       </c>
       <c r="D26" s="58" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E26" s="58" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F26" s="25"/>
       <c r="G26" s="58" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H26" s="35"/>
       <c r="I26"/>
@@ -1779,18 +1779,18 @@
         <v>3</v>
       </c>
       <c r="B27" s="52"/>
-      <c r="C27" s="63">
-        <v>2</v>
+      <c r="C27" s="57">
+        <v>3</v>
       </c>
       <c r="D27" s="58" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E27" s="58" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F27" s="25"/>
       <c r="G27" s="58" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="H27" s="35"/>
       <c r="I27"/>
@@ -1800,18 +1800,18 @@
         <v>3</v>
       </c>
       <c r="B28" s="52"/>
-      <c r="C28" s="63">
+      <c r="C28" s="57">
         <v>2</v>
       </c>
       <c r="D28" s="58" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E28" s="58" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F28" s="25"/>
       <c r="G28" s="58" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="H28" s="35"/>
       <c r="I28"/>
@@ -1820,19 +1820,19 @@
       <c r="A29" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B29" s="52"/>
-      <c r="C29" s="63">
-        <v>1</v>
+      <c r="B29" s="51"/>
+      <c r="C29" s="57">
+        <v>2</v>
       </c>
       <c r="D29" s="58" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E29" s="58" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F29" s="25"/>
       <c r="G29" s="58" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="H29" s="35"/>
       <c r="I29"/>
@@ -1841,19 +1841,19 @@
       <c r="A30" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B30" s="51"/>
-      <c r="C30" s="63">
+      <c r="B30" s="52"/>
+      <c r="C30" s="57">
         <v>1</v>
       </c>
       <c r="D30" s="58" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E30" s="58" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F30" s="25"/>
       <c r="G30" s="58" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="H30" s="35"/>
       <c r="I30"/>
@@ -1863,18 +1863,18 @@
         <v>3</v>
       </c>
       <c r="B31" s="52"/>
-      <c r="C31" s="63">
+      <c r="C31" s="57">
         <v>1</v>
       </c>
       <c r="D31" s="58" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E31" s="58" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F31" s="25"/>
       <c r="G31" s="58" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="H31" s="35"/>
       <c r="I31"/>
@@ -1883,19 +1883,19 @@
       <c r="A32" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B32" s="52"/>
-      <c r="C32" s="63">
+      <c r="B32" s="51"/>
+      <c r="C32" s="57">
         <v>1</v>
       </c>
       <c r="D32" s="58" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E32" s="58" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F32" s="25"/>
       <c r="G32" s="58" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="H32" s="35"/>
       <c r="I32"/>
@@ -1904,19 +1904,19 @@
       <c r="A33" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B33" s="51"/>
-      <c r="C33" s="63">
+      <c r="B33" s="52"/>
+      <c r="C33" s="57">
         <v>1</v>
       </c>
       <c r="D33" s="58" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E33" s="58" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F33" s="25"/>
       <c r="G33" s="58" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="H33" s="35"/>
       <c r="I33"/>
@@ -1926,18 +1926,18 @@
         <v>3</v>
       </c>
       <c r="B34" s="52"/>
-      <c r="C34" s="63">
+      <c r="C34" s="57">
         <v>1</v>
       </c>
       <c r="D34" s="58" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E34" s="58" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F34" s="25"/>
       <c r="G34" s="58" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="H34" s="35"/>
       <c r="I34"/>
@@ -1946,19 +1946,19 @@
       <c r="A35" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B35" s="52"/>
-      <c r="C35" s="63">
+      <c r="B35" s="51"/>
+      <c r="C35" s="57">
         <v>1</v>
       </c>
       <c r="D35" s="58" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E35" s="58" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F35" s="25"/>
       <c r="G35" s="58" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="H35" s="35"/>
       <c r="I35"/>
@@ -1967,19 +1967,19 @@
       <c r="A36" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B36" s="51"/>
-      <c r="C36" s="63">
+      <c r="B36" s="52"/>
+      <c r="C36" s="57">
         <v>1</v>
       </c>
       <c r="D36" s="58" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E36" s="58" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F36" s="25"/>
       <c r="G36" s="58" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="H36" s="35"/>
       <c r="I36"/>
@@ -1988,19 +1988,19 @@
       <c r="A37" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B37" s="52"/>
-      <c r="C37" s="63">
+      <c r="B37" s="51"/>
+      <c r="C37" s="57">
         <v>1</v>
       </c>
       <c r="D37" s="58" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E37" s="58" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F37" s="25"/>
       <c r="G37" s="58" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="H37" s="35"/>
       <c r="I37"/>
@@ -2010,18 +2010,18 @@
         <v>3</v>
       </c>
       <c r="B38" s="52"/>
-      <c r="C38" s="63">
+      <c r="C38" s="57">
         <v>1</v>
       </c>
       <c r="D38" s="58" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E38" s="58" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F38" s="25"/>
       <c r="G38" s="58" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="H38" s="35"/>
       <c r="I38"/>
@@ -2030,19 +2030,19 @@
       <c r="A39" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B39" s="51"/>
-      <c r="C39" s="63">
+      <c r="B39" s="52"/>
+      <c r="C39" s="57">
         <v>1</v>
       </c>
       <c r="D39" s="58" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E39" s="58" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="F39" s="25"/>
       <c r="G39" s="58" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="H39" s="35"/>
       <c r="I39"/>
@@ -2052,18 +2052,18 @@
         <v>3</v>
       </c>
       <c r="B40" s="52"/>
-      <c r="C40" s="63">
+      <c r="C40" s="57">
         <v>1</v>
       </c>
       <c r="D40" s="58" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E40" s="58" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F40" s="25"/>
-      <c r="G40" s="57" t="s">
-        <v>106</v>
+      <c r="G40" s="58" t="s">
+        <v>100</v>
       </c>
       <c r="H40" s="35"/>
       <c r="I40"/>
@@ -2072,7 +2072,7 @@
       <c r="A41" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B41" s="52"/>
+      <c r="B41" s="51"/>
       <c r="C41" s="63"/>
       <c r="D41" s="58"/>
       <c r="E41" s="58"/>
@@ -2082,9 +2082,7 @@
       <c r="I41"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="10" t="s">
-        <v>3</v>
-      </c>
+      <c r="A42" s="11"/>
       <c r="B42" s="52"/>
       <c r="C42" s="63"/>
       <c r="D42" s="58"/>
@@ -2095,10 +2093,8 @@
       <c r="I42"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B43" s="51"/>
+      <c r="A43" s="10"/>
+      <c r="B43" s="52"/>
       <c r="C43" s="63"/>
       <c r="D43" s="58"/>
       <c r="E43" s="58"/>
@@ -2108,8 +2104,8 @@
       <c r="I43"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="11"/>
-      <c r="B44" s="52"/>
+      <c r="A44" s="10"/>
+      <c r="B44" s="51"/>
       <c r="C44" s="63"/>
       <c r="D44" s="58"/>
       <c r="E44" s="58"/>
@@ -2131,7 +2127,7 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="10"/>
-      <c r="B46" s="51"/>
+      <c r="B46" s="52"/>
       <c r="C46" s="63"/>
       <c r="D46" s="58"/>
       <c r="E46" s="58"/>
@@ -2142,7 +2138,7 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="10"/>
-      <c r="B47" s="52"/>
+      <c r="B47" s="51"/>
       <c r="C47" s="63"/>
       <c r="D47" s="58"/>
       <c r="E47" s="58"/>
@@ -2164,7 +2160,7 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="10"/>
-      <c r="B49" s="51"/>
+      <c r="B49" s="52"/>
       <c r="C49" s="63"/>
       <c r="D49" s="58"/>
       <c r="E49" s="58"/>
@@ -2175,7 +2171,7 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="10"/>
-      <c r="B50" s="52"/>
+      <c r="B50" s="51"/>
       <c r="C50" s="63"/>
       <c r="D50" s="58"/>
       <c r="E50" s="58"/>
@@ -2197,7 +2193,7 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="10"/>
-      <c r="B52" s="51"/>
+      <c r="B52" s="52"/>
       <c r="C52" s="63"/>
       <c r="D52" s="58"/>
       <c r="E52" s="58"/>
@@ -2208,7 +2204,7 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="10"/>
-      <c r="B53" s="52"/>
+      <c r="B53" s="51"/>
       <c r="C53" s="63"/>
       <c r="D53" s="58"/>
       <c r="E53" s="58"/>
@@ -2230,7 +2226,7 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="10"/>
-      <c r="B55" s="51"/>
+      <c r="B55" s="52"/>
       <c r="C55" s="63"/>
       <c r="D55" s="58"/>
       <c r="E55" s="58"/>
@@ -2263,7 +2259,7 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="10"/>
-      <c r="B58" s="52"/>
+      <c r="B58" s="51"/>
       <c r="C58" s="63"/>
       <c r="D58" s="58"/>
       <c r="E58" s="58"/>
@@ -2285,7 +2281,7 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="10"/>
-      <c r="B60" s="51"/>
+      <c r="B60" s="52"/>
       <c r="C60" s="63"/>
       <c r="D60" s="58"/>
       <c r="E60" s="58"/>
@@ -2307,7 +2303,7 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="10"/>
-      <c r="B62" s="52"/>
+      <c r="B62" s="51"/>
       <c r="C62" s="63"/>
       <c r="D62" s="58"/>
       <c r="E62" s="58"/>
@@ -2351,7 +2347,7 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="10"/>
-      <c r="B66" s="51"/>
+      <c r="B66" s="52"/>
       <c r="C66" s="63"/>
       <c r="D66" s="58"/>
       <c r="E66" s="58"/>
@@ -2384,7 +2380,7 @@
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="10"/>
-      <c r="B69" s="52"/>
+      <c r="B69" s="51"/>
       <c r="C69" s="63"/>
       <c r="D69" s="58"/>
       <c r="E69" s="58"/>
@@ -2406,7 +2402,7 @@
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="10"/>
-      <c r="B71" s="51"/>
+      <c r="B71" s="52"/>
       <c r="C71" s="63"/>
       <c r="D71" s="58"/>
       <c r="E71" s="58"/>
@@ -2417,7 +2413,7 @@
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="10"/>
-      <c r="B72" s="52"/>
+      <c r="B72" s="51"/>
       <c r="C72" s="63"/>
       <c r="D72" s="58"/>
       <c r="E72" s="58"/>
@@ -2427,7 +2423,9 @@
       <c r="I72"/>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A73" s="10"/>
+      <c r="A73" s="10" t="s">
+        <v>3</v>
+      </c>
       <c r="B73" s="52"/>
       <c r="C73" s="63"/>
       <c r="D73" s="58"/>
@@ -2439,25 +2437,23 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="10"/>
-      <c r="B74" s="51"/>
-      <c r="C74" s="63"/>
-      <c r="D74" s="58"/>
-      <c r="E74" s="58"/>
+      <c r="B74" s="52"/>
+      <c r="C74" s="64"/>
+      <c r="D74" s="24"/>
+      <c r="E74" s="25"/>
       <c r="F74" s="25"/>
-      <c r="G74" s="58"/>
+      <c r="G74" s="50"/>
       <c r="H74" s="35"/>
       <c r="I74"/>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A75" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B75" s="52"/>
-      <c r="C75" s="63"/>
-      <c r="D75" s="58"/>
-      <c r="E75" s="58"/>
+      <c r="A75" s="10"/>
+      <c r="B75" s="51"/>
+      <c r="C75" s="64"/>
+      <c r="D75" s="24"/>
+      <c r="E75" s="25"/>
       <c r="F75" s="25"/>
-      <c r="G75" s="58"/>
+      <c r="G75" s="50"/>
       <c r="H75" s="35"/>
       <c r="I75"/>
     </row>
@@ -2474,7 +2470,7 @@
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" s="10"/>
-      <c r="B77" s="51"/>
+      <c r="B77" s="52"/>
       <c r="C77" s="64"/>
       <c r="D77" s="24"/>
       <c r="E77" s="25"/>
@@ -2485,7 +2481,7 @@
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="10"/>
-      <c r="B78" s="52"/>
+      <c r="B78" s="51"/>
       <c r="C78" s="64"/>
       <c r="D78" s="24"/>
       <c r="E78" s="25"/>
@@ -2507,7 +2503,7 @@
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="10"/>
-      <c r="B80" s="51"/>
+      <c r="B80" s="52"/>
       <c r="C80" s="64"/>
       <c r="D80" s="24"/>
       <c r="E80" s="25"/>
@@ -2518,7 +2514,7 @@
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" s="10"/>
-      <c r="B81" s="52"/>
+      <c r="B81" s="51"/>
       <c r="C81" s="64"/>
       <c r="D81" s="24"/>
       <c r="E81" s="25"/>
@@ -2540,7 +2536,7 @@
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" s="10"/>
-      <c r="B83" s="51"/>
+      <c r="B83" s="52"/>
       <c r="C83" s="64"/>
       <c r="D83" s="24"/>
       <c r="E83" s="25"/>
@@ -2551,7 +2547,7 @@
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" s="10"/>
-      <c r="B84" s="52"/>
+      <c r="B84" s="51"/>
       <c r="C84" s="64"/>
       <c r="D84" s="24"/>
       <c r="E84" s="25"/>
@@ -2573,7 +2569,7 @@
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="10"/>
-      <c r="B86" s="51"/>
+      <c r="B86" s="52"/>
       <c r="C86" s="64"/>
       <c r="D86" s="24"/>
       <c r="E86" s="25"/>
@@ -2584,7 +2580,7 @@
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" s="10"/>
-      <c r="B87" s="52"/>
+      <c r="B87" s="51"/>
       <c r="C87" s="64"/>
       <c r="D87" s="24"/>
       <c r="E87" s="25"/>
@@ -2606,7 +2602,7 @@
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" s="10"/>
-      <c r="B89" s="51"/>
+      <c r="B89" s="52"/>
       <c r="C89" s="64"/>
       <c r="D89" s="24"/>
       <c r="E89" s="25"/>
@@ -2617,7 +2613,7 @@
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" s="10"/>
-      <c r="B90" s="52"/>
+      <c r="B90" s="51"/>
       <c r="C90" s="64"/>
       <c r="D90" s="24"/>
       <c r="E90" s="25"/>
@@ -2639,7 +2635,7 @@
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" s="10"/>
-      <c r="B92" s="51"/>
+      <c r="B92" s="52"/>
       <c r="C92" s="64"/>
       <c r="D92" s="24"/>
       <c r="E92" s="25"/>
@@ -2650,7 +2646,7 @@
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" s="10"/>
-      <c r="B93" s="52"/>
+      <c r="B93" s="51"/>
       <c r="C93" s="64"/>
       <c r="D93" s="24"/>
       <c r="E93" s="25"/>
@@ -2659,52 +2655,30 @@
       <c r="H93" s="35"/>
       <c r="I93"/>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A94" s="10"/>
-      <c r="B94" s="52"/>
-      <c r="C94" s="64"/>
-      <c r="D94" s="24"/>
-      <c r="E94" s="25"/>
-      <c r="F94" s="25"/>
-      <c r="G94" s="50"/>
-      <c r="H94" s="35"/>
+      <c r="B94" s="56"/>
+      <c r="C94" s="65"/>
+      <c r="D94" s="53"/>
+      <c r="E94" s="54"/>
+      <c r="F94" s="54"/>
+      <c r="G94" s="55"/>
+      <c r="H94" s="36"/>
       <c r="I94"/>
+      <c r="J94"/>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A95" s="10"/>
-      <c r="B95" s="51"/>
-      <c r="C95" s="64"/>
-      <c r="D95" s="24"/>
-      <c r="E95" s="25"/>
-      <c r="F95" s="25"/>
-      <c r="G95" s="50"/>
-      <c r="H95" s="35"/>
-      <c r="I95"/>
-    </row>
-    <row r="96" spans="1:10" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="10"/>
-      <c r="B96" s="56"/>
-      <c r="C96" s="65"/>
-      <c r="D96" s="53"/>
-      <c r="E96" s="54"/>
-      <c r="F96" s="54"/>
-      <c r="G96" s="55"/>
-      <c r="H96" s="36"/>
-      <c r="I96"/>
-      <c r="J96"/>
-    </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A97" s="28"/>
-      <c r="B97" s="28"/>
-      <c r="C97" s="66">
-        <f>SUM(C10:C96)</f>
-        <v>44</v>
-      </c>
-      <c r="D97" s="29"/>
-      <c r="E97" s="30"/>
-      <c r="F97" s="29"/>
-      <c r="G97" s="31"/>
-      <c r="H97" s="32"/>
+      <c r="A95" s="28"/>
+      <c r="B95" s="28"/>
+      <c r="C95" s="66">
+        <f>SUM(C10:C94)</f>
+        <v>43</v>
+      </c>
+      <c r="D95" s="29"/>
+      <c r="E95" s="30"/>
+      <c r="F95" s="29"/>
+      <c r="G95" s="31"/>
+      <c r="H95" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>